<commit_message>
feat: tailor outputs for lawyer review
</commit_message>
<xml_diff>
--- a/examples/demo-labor-dispute/result-sample/整理结果/案件材料汇总.xlsx
+++ b/examples/demo-labor-dispute/result-sample/整理结果/案件材料汇总.xlsx
@@ -8,19 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件概览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料清单" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件时间轴" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当事人信息" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="音视频材料" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="案件时间轴" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题与待补材料" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="材料清单" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待补材料" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'案件概览'!$A$3:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'材料清单'!$A$3:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'案件时间轴'!$A$3:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'当事人信息'!$A$3:$D$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'音视频材料'!$A$3:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'案件时间轴'!$A$3:$E$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'问题与待补材料'!$A$3:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'材料清单'!$A$3:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'待补材料'!$A$3:$D$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
+          <t>律师阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
@@ -584,28 +582,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>材料清单</t>
+          <t>案件时间轴</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
+          <t>律师阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
@@ -617,419 +614,219 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>材料名称</t>
+          <t>事件</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>材料类型</t>
+          <t>相关人员/公司</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>主要内容</t>
+          <t>相关材料</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>所在文件夹</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>处理状态</t>
+          <t>待确认事项</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>2024-03-12</t>
+          <t>2023-03-06</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>240312-林晚晴_私聊_加班未结算.png</t>
+          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>图片</t>
+          <t>沪江优配仓储服务有限公司（演示）等合作主体</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
+          <t>230306-仓配服务与用工管理总协议.docx</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>协议附件、盖章和具体责任边界仍待核。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2024-08-30</t>
+          <t>2023-04-10</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>240830-高雪_私聊_工资扣款.png</t>
+          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>图片</t>
+          <t>林晚晴；沪江优配仓储服务有限公司（演示）</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
+          <t>230410-林晚晴_E001_劳动合同.docx；时间待核-案件当事人初始情况说明.txt</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>实际管理、发薪和社保主体需结合其他材料核对。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>2024-07-22</t>
+          <t>2024-03-08至2024-03-10</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>240722-孙浩_现场事故记录.docx</t>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Word文档</t>
+          <t>林晚晴；现场主管</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
+          <t>240312-林晚晴_私聊_加班未结算.png；2403-林晚晴_工资条拍照件.jpg；2403-林晚晴_银行转账详情.png</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>仍需原始考勤、排班和加班审批记录逐笔核对。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>2023-04-10</t>
+          <t>2024-07-22</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>230410-林晚晴_E001_劳动合同.docx</t>
+          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>合同</t>
+          <t>孙浩；现场主管</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
+          <t>240722-孙浩_现场事故记录.docx；240722-孙浩_现场设备照片.jpg</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>设备状态、现场人员和事故申报情况待核。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2025-03-05</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>250305-工资支付延期说明.txt</t>
+          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>文本材料</t>
+          <t>孙浩</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
+          <t>240723-孙浩_门诊凭证照片.jpg</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>票据原件、伤情和工伤关联性待核。</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-08-30</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2403-林晚晴_工资条拍照件.jpg</t>
+          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>图片</t>
+          <t>高雪；HR；财务</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
+          <t>2408-高雪_工资条拍照件.jpg；240830-高雪_私聊_工资扣款.png</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>原始考勤、扣款计算和员工确认缺失。</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>时间待确认</t>
+          <t>2025-03-05</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>时间待核-案件当事人初始情况说明.txt</t>
+          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>主体/工商材料</t>
+          <t>沪江优配仓储服务有限公司（演示）；相关员工</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
+          <t>250305-工资支付延期说明.txt</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>001 主体信息</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>2023-03-06</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>230306-仓配服务与用工管理总协议.docx</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>协议</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>2024-07-22</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>240722-孙浩_现场设备照片.jpg</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>图片/照片</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>2024-03</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>2403-林晚晴_银行转账详情.png</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>转账记录</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>240723-孙浩_门诊凭证照片.jpg</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>图片/照片</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>2024-08</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>2408-高雪_工资条拍照件.jpg</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>图片</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>002 基础资料</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>已读取</t>
+          <t>原说明、盖章状态和实际支付金额待核。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F15"/>
+  <autoFilter ref="A3:E10"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1060,7 +857,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
+          <t>律师阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
@@ -1190,318 +987,458 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>音视频材料</t>
+          <t>材料清单</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
+          <t>律师阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>文件名称</t>
+          <t>日期</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>对应逐字稿</t>
+          <t>材料名称</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>处理情况</t>
+          <t>材料类型</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>主要内容</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>所在文件夹</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>处理状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2024-03-12</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>240312-林晚晴_私聊_加班未结算.png</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>图片</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>2024-08-30</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>240830-高雪_私聊_工资扣款.png</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>图片</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2024-07-22</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>240722-孙浩_现场事故记录.docx</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Word文档</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>2023-04-10</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>230410-林晚晴_E001_劳动合同.docx</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>合同</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2025-03-05</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>250305-工资支付延期说明.txt</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>文本材料</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2403-林晚晴_工资条拍照件.jpg</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>图片</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>时间待确认</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>时间待核-案件当事人初始情况说明.txt</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>主体/工商材料</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>001 主体信息</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>2023-03-06</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>230306-仓配服务与用工管理总协议.docx</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>协议</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2024-07-22</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>240722-孙浩_现场设备照片.jpg</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>图片/照片</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2403-林晚晴_银行转账详情.png</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>转账记录</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2024-07-23</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>240723-孙浩_门诊凭证照片.jpg</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>图片/照片</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2408-高雪_工资条拍照件.jpg</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>图片</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>002 基础资料</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>已整理</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D3"/>
+  <autoFilter ref="A3:F15"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>案件时间轴</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>日期</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>事件</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>相关人员/公司</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>相关材料</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>待确认事项</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>2023-03-06</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>协议材料记载有关主体形成仓配服务和用工管理合作安排。</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>沪江优配仓储服务有限公司（演示）等合作主体</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>230306-仓配服务与用工管理总协议.docx</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>协议附件、盖章和具体责任边界仍待核。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>2023-04-10</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>劳动合同记载林晚晴以仓库拣货员岗位入职。</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>林晚晴；沪江优配仓储服务有限公司（演示）</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>230410-林晚晴_E001_劳动合同.docx；时间待核-案件当事人初始情况说明.txt</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>实际管理、发薪和社保主体需结合其他材料核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>2024-03-08至2024-03-10</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>聊天和薪资材料记载盘点期间延长工作，林晚晴提出加班未结算。</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>林晚晴；现场主管</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>240312-林晚晴_私聊_加班未结算.png；2403-林晚晴_工资条拍照件.jpg；2403-林晚晴_银行转账详情.png</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>仍需原始考勤、排班和加班审批记录逐笔核对。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2024-07-22</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>事故记录和现场照片记载孙浩处理卡料时手部受伤。</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>孙浩；现场主管</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>240722-孙浩_现场事故记录.docx；240722-孙浩_现场设备照片.jpg</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>设备状态、现场人员和事故申报情况待核。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>2024-07-23</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>门诊凭证记载孙浩事故后就诊并发生医疗支出。</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>孙浩</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>240723-孙浩_门诊凭证照片.jpg</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>票据原件、伤情和工伤关联性待核。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>2024-08-30</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>工资条和聊天记载高雪8月工资因异常考勤扣减680元，高雪提出异议。</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>高雪；HR；财务</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>2408-高雪_工资条拍照件.jpg；240830-高雪_私聊_工资扣款.png</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>原始考勤、扣款计算和员工确认缺失。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>2025-03-05</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>延期说明称部分工资和补贴因客户结算延迟而顺延。</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>沪江优配仓储服务有限公司（演示）；相关员工</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>250305-工资支付延期说明.txt</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>原说明、盖章状态和实际支付金额待核。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:E10"/>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1519,14 +1456,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>问题与待补材料</t>
+          <t>待补材料</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>用户阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
+          <t>律师阅读版：仅展示理解案件所需信息；不确定内容统一标记为‘待确认’。</t>
         </is>
       </c>
     </row>

</xml_diff>